<commit_message>
v2d: C46 back to the 220u/25V polymer (C2981459), C44 to 10u/50V (C53084452)
A stale 'C44-C47 = 22u/25V 1210' line in the generator's LCSC table
overrode both: C46 became a 22u ceramic (the LM3150 needs the polymer's
ESR) and C44, on VIN up to 26 V, a 25 V part. Caught in JLC's matching sheet.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radio_Kiosk_v2d/fab/v2d-bom-jlc-smt.xlsx
+++ b/Radio_Kiosk_v2d/fab/v2d-bom-jlc-smt.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D103"/>
+  <dimension ref="A1:D102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -666,7 +666,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>C30,C40,C50,C90,C91</t>
+          <t>C30,C40,C50,C90,C91,C44</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -793,78 +793,78 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10u/50V</t>
+          <t>220u/25V polymer</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>C44</t>
+          <t>C46</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>C_1210_3225Metric</t>
+          <t>CP_Elec_6.3x7.7</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>C53084530</t>
+          <t>C2981459</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>220u/25V polymer</t>
+          <t>2.2n</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>C46</t>
+          <t>C49</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CP_Elec_6.3x7.7</t>
+          <t>C_0805_2012Metric</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C53084530</t>
+          <t>C28260</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2.2n</t>
+          <t>1u/100V</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>C49</t>
+          <t>C62,C70</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>C_0805_2012Metric</t>
+          <t>C_1210_3225Metric</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>C28260</t>
+          <t>C24365</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1u/100V</t>
+          <t>220n/100V</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>C62,C70</t>
+          <t>C71</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -874,63 +874,63 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>C24365</t>
+          <t>C72067</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>220n/100V</t>
+          <t>470u/25V</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>C71</t>
+          <t>C97,C98</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>C_1210_3225Metric</t>
+          <t>CP_Elec_10x10.5</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>C72067</t>
+          <t>C346948</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>470u/25V</t>
+          <t>4.7n</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>C97,C98</t>
+          <t>C117</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CP_Elec_10x10.5</t>
+          <t>C_0805_2012Metric</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>C346948</t>
+          <t>C1744</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>4.7n</t>
+          <t>4.7u</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>C117</t>
+          <t>C130</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -940,41 +940,41 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>C1744</t>
+          <t>C1779</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4.7u</t>
+          <t>1u</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>C130</t>
+          <t>C141</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>C_0805_2012Metric</t>
+          <t>C_0603_1608Metric</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>C1779</t>
+          <t>C15849</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1u</t>
+          <t>10u</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>C141</t>
+          <t>C142,C143</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -984,41 +984,41 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>C15849</t>
+          <t>C19702</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>SMAJ22A TVS</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>C142,C143</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>C_0603_1608Metric</t>
+          <t>D_SMA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>C19702</t>
+          <t>C148220</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SMAJ22A TVS</t>
+          <t>SMAJ28A TVS</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1028,19 +1028,19 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>C148220</t>
+          <t>C148227</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SMAJ28A TVS</t>
+          <t>SS310 100V Schottky</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1050,107 +1050,107 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>C148227</t>
+          <t>C15874</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SS310 100V Schottky</t>
+          <t>1N4148W</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D21,D40</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>D_SMA</t>
+          <t>D_SOD-123</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>C15874</t>
+          <t>C81598</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1N4148W</t>
+          <t>SMAJ58A TVS</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>D21,D40</t>
+          <t>D22,D70</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>D_SOD-123</t>
+          <t>D_SMA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>C81598</t>
+          <t>C10762</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SMAJ58A TVS</t>
+          <t>BZT52C12 zener</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>D22,D70</t>
+          <t>D23,D24</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>D_SMA</t>
+          <t>D_SOD-123</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>C10762</t>
+          <t>C12747</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BZT52C12 zener</t>
+          <t>WS2812B-4020 power LED</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>D23,D24</t>
+          <t>D30</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>D_SOD-123</t>
+          <t>LED-SMD_WS2812B-4020</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>C12747</t>
+          <t>C965557</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>WS2812B-4020 power LED</t>
+          <t>WS2812B-4020 radio LED</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>D30</t>
+          <t>D31</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1167,34 +1167,34 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>WS2812B-4020 radio LED</t>
+          <t>SS14 flyback</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>D31</t>
+          <t>D32</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LED-SMD_WS2812B-4020</t>
+          <t>D_SMA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>C965557</t>
+          <t>C2480</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SS14 flyback</t>
+          <t>S1B clamp</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>D32</t>
+          <t>D71</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1204,68 +1204,68 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>C2480</t>
+          <t>C96324</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>S1B clamp</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>D71</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>D_SMA</t>
+          <t>Fuse_1206_3216Metric</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>C96324</t>
+          <t>C2838912</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>USB-C PD in</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Fuse_1206_3216Metric</t>
+          <t>USB-C_TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>C2838912</t>
+          <t>C165948</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>USB-C PD in</t>
+          <t>USB-C</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J12</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>USB-C_TYPE-C-31-M-12</t>
+          <t>USB_C_Receptacle_HRO_TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1277,144 +1277,144 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>USB-C</t>
+          <t>MDA1040-150M 15u 6A</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>J12</t>
+          <t>L3,L4</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>USB_C_Receptacle_HRO_TYPE-C-31-M-12</t>
+          <t>IND-SMD_L10.0-W10.0-APS10A40M470</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>C165948</t>
+          <t>C2847554</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MDA1040-150M 15u 6A</t>
+          <t>SRP7028A-100M 10u 3.5A</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>L3,L4</t>
+          <t>L5</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>IND-SMD_L10.0-W10.0-APS10A40M470</t>
+          <t>L_Bourns_SRP7028A_7.3x6.6mm</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>C2847554</t>
+          <t>C2687402</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SRP7028A-100M 10u 3.5A</t>
+          <t>MDA1365-330M 33u 9A</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>L5</t>
+          <t>L20</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>L_Bourns_SRP7028A_7.3x6.6mm</t>
+          <t>L_12x12mm_H8mm</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>C2687402</t>
+          <t>C2847586</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MDA1365-330M 33u 9A</t>
+          <t>SI4470EY</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>L20</t>
+          <t>Q1,Q2,Q6,Q7,Q12</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>L_12x12mm_H8mm</t>
+          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>C2847586</t>
+          <t>C7568913</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SI4470EY</t>
+          <t>AOD4185</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Q1,Q2,Q6,Q7,Q12</t>
+          <t>Q8</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>TO-252-2</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>C7568913</t>
+          <t>C400894</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AOD4185</t>
+          <t>2N7002</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Q8</t>
+          <t>Q9,Q10,Q25,Q45</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>TO-252-2</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>C400894</t>
+          <t>C8545</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2N7002</t>
+          <t>AO3400A</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Q9,Q10,Q25,Q45</t>
+          <t>Q11,Q30</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1424,173 +1424,173 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>C8545</t>
+          <t>C20917</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>AO3400A</t>
+          <t>AO4482</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Q11,Q30</t>
+          <t>Q13,Q20</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>C20917</t>
+          <t>C192576</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>AO4482</t>
+          <t>PSMN075-100MSEX</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Q13,Q20</t>
+          <t>Q22</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>LFPAK33</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>C192576</t>
+          <t>C478016</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PSMN075-100MSEX</t>
+          <t>DMP10H400SE</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Q22</t>
+          <t>Q23</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>LFPAK33</t>
+          <t>SOT-223_L6.5-W3.5-P2.30-LS7.0-BR</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>C478016</t>
+          <t>C156277</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DMP10H400SE</t>
+          <t>BSS123</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Q23</t>
+          <t>Q24</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SOT-223_L6.5-W3.5-P2.30-LS7.0-BR</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>C156277</t>
+          <t>C78755</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BSS123</t>
+          <t>AOD4184A</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Q24</t>
+          <t>Q40,Q41</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>TO-252-2</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>C78755</t>
+          <t>C99124</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>AOD4184A</t>
+          <t>SI4401DDY</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Q40,Q41</t>
+          <t>Q44</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>TO-252-2</t>
+          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>C99124</t>
+          <t>C72317</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SI4401DDY</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Q44</t>
+          <t>R5,R6,R29,R42,R80,R89,R92,R97,R100,R101</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>C72317</t>
+          <t>C149504</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>R5,R6,R29,R42,R80,R89,R92,R97,R100,R101</t>
+          <t>R7,R9,R24,R26,R27,R46,R47,R49,R61,R62,R63,R66,R78,R79,R82,R83,R99,R105,R107,R111,R121</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1600,19 +1600,19 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>C149504</t>
+          <t>C17414</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>47k</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>R7,R9,R24,R26,R27,R46,R47,R49,R61,R62,R63,R66,R78,R79,R82,R83,R99,R105,R107,R111,R121</t>
+          <t>R8,R21,R28,R48</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1622,19 +1622,19 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>C17414</t>
+          <t>C17713</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>47k</t>
+          <t>20k</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>R8,R21,R28,R48</t>
+          <t>R10,R31</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1644,63 +1644,63 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>C17713</t>
+          <t>C4328</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>20k</t>
+          <t>15m 1W</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>R10,R31</t>
+          <t>R20</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>C4328</t>
+          <t>C44883</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>15m 1W</t>
+          <t>499k 1%</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>R20</t>
+          <t>R22</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>C44883</t>
+          <t>C17721</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>499k 1%</t>
+          <t>12k</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>R22</t>
+          <t>R23,R50</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1710,19 +1710,19 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>C17721</t>
+          <t>C17444</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>12k</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>R23,R50</t>
+          <t>R25,R81</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1732,19 +1732,19 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>C17444</t>
+          <t>C17513</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>220k</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>R25,R81</t>
+          <t>R30</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1754,19 +1754,19 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>C17513</t>
+          <t>C17556</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>220k</t>
+          <t>2k</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>R30</t>
+          <t>R40</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1776,19 +1776,19 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>C17556</t>
+          <t>C17604</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2k</t>
+          <t>51k</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>R40</t>
+          <t>R41,R65</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1798,19 +1798,19 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>C17604</t>
+          <t>C17737</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>51k</t>
+          <t>820k</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>R41,R65</t>
+          <t>R44</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1820,19 +1820,19 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>C17737</t>
+          <t>C50136</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>820k</t>
+          <t>750R</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>R44</t>
+          <t>R45</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1842,19 +1842,19 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>C50136</t>
+          <t>C17818</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>750R</t>
+          <t>3k</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>R45</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1864,19 +1864,19 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>C17818</t>
+          <t>C17661</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>3k</t>
+          <t>5.6k</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>R51</t>
+          <t>R60</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1886,19 +1886,19 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>C17661</t>
+          <t>C4382</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>5.6k</t>
+          <t>1M 1%</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>R60</t>
+          <t>R64,R86</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1908,19 +1908,19 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>C4382</t>
+          <t>C17514</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>1M 1%</t>
+          <t>10R</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>R64,R86</t>
+          <t>R70</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1930,19 +1930,19 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>C17514</t>
+          <t>C17415</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>10R</t>
+          <t>200R</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>R70</t>
+          <t>R71</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1952,63 +1952,63 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>C17415</t>
+          <t>C17540</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>200R</t>
+          <t>0.1R 1% 2W</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>R71</t>
+          <t>R72</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>C17540</t>
+          <t>C844904</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>0.1R 1% 2W</t>
+          <t>3.3k</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>R72</t>
+          <t>R73</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>C844904</t>
+          <t>C26010</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>3.3k</t>
+          <t>100R</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>R73</t>
+          <t>R74,R75,R76,R77,R103,R106</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2018,19 +2018,19 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>C26010</t>
+          <t>C17408</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>100R</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>R74,R75,R76,R77,R103,R106</t>
+          <t>R84</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2040,63 +2040,63 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>C17408</t>
+          <t>C17514</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>24R 2W pulse</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>R84</t>
+          <t>R85,R88</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>C17514</t>
+          <t>C25476</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>24R 2W pulse</t>
+          <t>150k</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>R85,R88</t>
+          <t>R87</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>C25476</t>
+          <t>C17470</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>150k</t>
+          <t>33k</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>R87</t>
+          <t>R90,R94</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2106,19 +2106,19 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>C17470</t>
+          <t>C17633</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>33k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>R90,R94</t>
+          <t>R91,R95,R98</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2128,63 +2128,63 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>C17633</t>
+          <t>C17673</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>20m 1W</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>R91,R95,R98</t>
+          <t>R93,R96</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>C17673</t>
+          <t>C2885416</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>20m 1W</t>
+          <t>1R</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>R93,R96</t>
+          <t>R104</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>C2885416</t>
+          <t>C25271</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>1R</t>
+          <t>0R</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>R104</t>
+          <t>R112</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2194,19 +2194,19 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>C25271</t>
+          <t>C17477</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>0R</t>
+          <t>220R</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>R112</t>
+          <t>R113</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2216,19 +2216,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>C17477</t>
+          <t>C17557</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>220R</t>
+          <t>120k 1%</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>R113</t>
+          <t>R120</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2238,41 +2238,41 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>C17557</t>
+          <t>C17436</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>120k 1%</t>
+          <t>5.1k</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>R120</t>
+          <t>R122,R123</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_0603_1608Metric</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>C17436</t>
+          <t>C23186</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>5.1k</t>
+          <t>10k NTC</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>R122,R123</t>
+          <t>RT1</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2282,41 +2282,41 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>C23186</t>
+          <t>C13564</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>10k NTC</t>
+          <t>RESET</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>RT1</t>
+          <t>SW1</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>SW_SPST_B3U-1000P</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>C13564</t>
+          <t>C231329</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>RESET</t>
+          <t>BOOT0 (DFU)</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SW1</t>
+          <t>SW2</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2333,254 +2333,254 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>BOOT0 (DFU)</t>
+          <t>LM74700-Q1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SW2</t>
+          <t>U1,U2,U6,U7,U12</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>SW_SPST_B3U-1000P</t>
+          <t>SOT-23-6</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>C231329</t>
+          <t>C2941042</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>LM74700-Q1</t>
+          <t>LMR33630 12V</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>U1,U2,U6,U7,U12</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>SOT-23-6</t>
+          <t>SOIC-8-1EP_3.9x4.9mm_P1.27mm_EP2.29x3mm</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>C2941042</t>
+          <t>C841384</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>LMR33630 12V</t>
+          <t>LM3150 15.75V 4.5A</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>SOIC-8-1EP_3.9x4.9mm_P1.27mm_EP2.29x3mm</t>
+          <t>HTSSOP-14_L5.0-W4.4-P0.65-LS6.4-BL-EP</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>C841384</t>
+          <t>C48112</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>LM3150 15.75V 4.5A</t>
+          <t>LMR33630 5V</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>U4</t>
+          <t>U5</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>HTSSOP-14_L5.0-W4.4-P0.65-LS6.4-BL-EP</t>
+          <t>SOIC-8-1EP_3.9x4.9mm_P1.27mm_EP2.29x3mm</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>C48112</t>
+          <t>C841384</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>LMR33630 5V</t>
+          <t>TLV7011</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>U10,U45</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>SOIC-8-1EP_3.9x4.9mm_P1.27mm_EP2.29x3mm</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>C841384</t>
+          <t>C702117</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>TLV7011</t>
+          <t>LM3478 54V boost</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>U10,U45</t>
+          <t>U20</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>C702117</t>
+          <t>C115907</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>LM3478 54V boost</t>
+          <t>TPS26600 eFuse</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>U20</t>
+          <t>U21</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>HTSSOP-16-1EP_4.4x5mm_P0.65mm_EP3.4x5mm</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>C115907</t>
+          <t>C544399</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>TPS26600 eFuse</t>
+          <t>LTC4279</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>U21</t>
+          <t>U22</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>HTSSOP-16-1EP_4.4x5mm_P0.65mm_EP3.4x5mm</t>
+          <t>SOIC-16_3.9x9.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>C544399</t>
+          <t>C687935</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>LTC4279</t>
+          <t>SN74AHCT1G125</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>U22</t>
+          <t>U30,U31</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>SOIC-16_3.9x9.9mm_P1.27mm</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>C687935</t>
+          <t>C7484</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SN74AHCT1G125</t>
+          <t>STM32F072CBT6</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>U30,U31</t>
+          <t>U40</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>LQFP-48_7x7mm_P0.5mm</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>C7484</t>
+          <t>C81720</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>STM32F072CBT6</t>
+          <t>INA180A1</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>U40</t>
+          <t>U41,U42</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>LQFP-48_7x7mm_P0.5mm</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>C81720</t>
+          <t>C122228</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>INA180A1</t>
+          <t>MCP6001T-I/OT</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>U41,U42</t>
+          <t>U43</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2590,93 +2590,71 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>C122228</t>
+          <t>C116490</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>MCP6001T-I/OT</t>
+          <t>CH224A</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>U43</t>
+          <t>U50</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>ESSOP-10_CH224A</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>C116490</t>
+          <t>C42459160</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CH224A</t>
+          <t>AP2112K-3.3</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>U50</t>
+          <t>U51</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ESSOP-10_CH224A</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>C42459160</t>
+          <t>C51118</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>AP2112K-3.3</t>
+          <t>USBLC6-2SC6</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>U51</t>
+          <t>U52</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>SOT-23-6</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
-        <is>
-          <t>C51118</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>USBLC6-2SC6</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>U52</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>SOT-23-6</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
         <is>
           <t>C7519</t>
         </is>

</xml_diff>